<commit_message>
further cell naming and dairy enteric test setup
</commit_message>
<xml_diff>
--- a/Excel/14_Electricity_Scope2_WIP_v02.xlsx
+++ b/Excel/14_Electricity_Scope2_WIP_v02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8013309D-5381-48B8-A506-3B26B735A5AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61A1EAF4-C5C2-41CF-829B-2D8D67A18BFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="465" windowWidth="35745" windowHeight="18900" firstSheet="2" activeTab="4" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="1755" yWindow="1020" windowWidth="36255" windowHeight="19140" firstSheet="2" activeTab="4" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -269,6 +269,7 @@
     <definedName name="X_Cell_Electricity_Market_AmountPurchasedGreenPower">'Input - Electricity'!$E$27</definedName>
     <definedName name="X_Cell_Electricity_Market_JurisdictionalRenewablePowerPercentage">'Input - Electricity'!$E$25</definedName>
     <definedName name="X_Cell_Electricity_Market_RenewablePowerPercentage">'Input - Electricity'!$E$24</definedName>
+    <definedName name="X_Cell_Site_EndDate">'Input - Site'!$E$13</definedName>
     <definedName name="X_Cell_Site_FarmName">'Input - Site'!$E$7</definedName>
     <definedName name="X_Cell_Site_Region">'Input - Site'!$E$22</definedName>
     <definedName name="X_Cell_Site_ReportingEntityName">'Input - Site'!$E$8</definedName>
@@ -8171,7 +8172,7 @@
         <v>91</v>
       </c>
       <c r="E16" s="29" t="str">
-        <f>IF('Input - Site'!E21="Western Australia", 'Input - Site'!E22, 'Input - Site'!E21)</f>
+        <f>IF(X_Cell_Site_State="Western Australia", X_Cell_Site_Region, X_Cell_Site_State)</f>
         <v>Western Australia - Outback (South)</v>
       </c>
       <c r="F16" s="19"/>
@@ -8265,7 +8266,7 @@
         <v>142</v>
       </c>
       <c r="E29" s="116" t="str">
-        <f>TEXT('Input - Site'!$E$12, "dd mmm yyyy")</f>
+        <f>TEXT('Input - Site'!E12, "dd mmm yyyy")</f>
         <v>01 Jan 2024</v>
       </c>
       <c r="K29" s="49"/>
@@ -8276,7 +8277,7 @@
         <v>127</v>
       </c>
       <c r="E30" s="116" t="str">
-        <f>TEXT('Input - Site'!$E$13, "dd mmm yyyy")</f>
+        <f>TEXT('Input - Site'!E13, "dd mmm yyyy")</f>
         <v>31 Dec 2024</v>
       </c>
       <c r="K30" s="49"/>
@@ -13946,10 +13947,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACkAKgAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADIAKQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlACkAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwBlAGwAbAAsACAARABlAGwAaQBtAGkAdABlAHIALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEAXQAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgBdACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgBYAE0ATAAoAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAHQAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMAcwBcAHUAMAAwADMAZQBcACIAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFMAVQBCAFMAVABJAFQAVQBUAEUAKABDAGUAbABsACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEALABcACIAXAAiACkALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABEAGUAbABpAG0AaQB0AGUAcgAsAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMAcwBcAHUAMAAwADMAZQBcACIAXABuACAAIAAgACAAIAAgACAAIAApACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAC8AdABcAHUAMAAwADMAZQBcACIALABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAvAC8AcwBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAGEAdgBnAFQAZQBtAHAALABhAHYAZwBSAGEAaQBuACwAZgByAG8AcwB0AEQAYQB5AHMALABlAGwAZQB2ACwAbQBhAHAAXwBwAGUAdAAsAFwAbgAgACAAIAAgAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACwAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkALABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUABFAFQAQQByAHIAYQB5ACwAbQBhAHgAUABFAFQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AG0AYQBwAF8AcABlAHQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABQAEUAVABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AG0AYQBwAF8AcABlAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABBAEsARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgADEAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAE0AaQBuAEEAcgByAGEAeQAsACAATQBhAHgAQQByAHIAYQB5ACwAIABJAHQAZQBtAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AaQBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABJAHQAZQBtAEEAcgByAGEAeQAsACAAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAQwByAGkAdABlAHIAaQBhADEALAAgAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5ACwAIABRAHUAYQBuAHQAaQB0AHkALAAgAFsATQB1AGwAdABpAHAAbABpAGUAcgBdACwAIABbAEMAcgBpAHQAZQByAGkAYQAyAF0ALABbAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQBdACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgATQB1AGwAdABpAHAAbABpAGUAcgApACwAMQAsAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsAFwAbgAgACAAIAAgAHEAdQBhAG4AdABpAHQAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACoATQB1AGwAdABpAHAAbABpAGUAcgAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMQApACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADIALABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAcgBpAHQAZQByAGkAYQAyACkALAAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADIAKQApACwAXABuACAAIAAgACAAUwBVAE0AUABSAE8ARABVAEMAVAAoAGMAcgBpAHQAZQByAGkAYQAxACoAYwByAGkAdABlAHIAaQBhADIAKgBxAHUAYQBuAHQAaQB0AHkAKQBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjACAAUwApACwAXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAG4AZQB4AHQAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAUwApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBiACAAcwB0AGEAcgB0AHMAIABhAGYAdABlAHIAIABFACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUARQApACwAXABuACAAIAAgACAAIAAgACAAIABuACwATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAcgBzACwAUwBFAFEAVQBFAE4AQwBFACgAbgAsADEALABmAGkAcgBzAHQAWQBlAGEAcgAsADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMALABEAEEAVABFACgAeQByAHMALABtACwAZAApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzACwATQBBAFAAKABzAHQAYQByAHQAcwAsAFAAZQByAGkAbwBkAEUAbgBkACkALABcAG4AIAAgACAAIAAgACAAIAAgAHQAYQBnACwASQBGACgAcwB0AGEAcgB0AHMAPQBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXAAiACAAKABUAGgAaQBzACAAcgBlAHAAbwByAHQAaQBuAGcAIABjAHkAYwBsAGUAKQBcACIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzAFQAZQB4AHQALABUAEUAWABUACgAcwB0AGEAcgB0AHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzAFQAZQB4AHQALABUAEUAWABUACgAZQBuAGQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAXAAiACAAdABvACAAXAAiACAAXAB1ADAAMAAyADYAIABlAG4AZABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAHQAYQBnACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQBcAG4APQBMAEEATQBCAEQAQQAoAEYAdQBuAGMAdABpAG8AbgAsACAAVABFAFgAVABCAEUARgBPAFIARQAoAEYATwBSAE0AVQBMAEEAVABFAFgAVAAoAEYAdQBuAGMAdABpAG8AbgApACwAIABcACIAKABcACIAKQApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5ACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkALABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAA9AFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACAAPQAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5AD0AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkAPQBJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkAPQBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAFwAdQAwADAAMwBlADAALAAgADEALAAgADAAKQBcAG4AIAAgACAAIAApACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAdQAwADAAMgA3AFwAIgAgAFwAdQAwADAAMgA2ACAAcwBoACAAXAB1ADAAMAAyADYAIABcACIAXAB1ADAAMAAyADcAIQBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsARABpAGYAZgBlAHIAZQBuAHQAUwBoAGUAZQB0AFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAxAF8AMgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADEALAAgADIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADMALAAgADQAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAATQBNAFMALAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFwAbgAgACAAIAAgACAAIAAgACAATQBFAEQASQBBAE4AKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ASQBuAGQAaQByAGUAYwB0ACAAKABzAGMAbwBwAGUAIAAyACAAYQBuAGQAIABzAGMAbwBwAGUAIAAzACkAIABsAG8AYwBhAHQAaQBvAG4ALQBiAGEAcwBlAGQAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAYQBzAHMAbwBjAGkAYQB0AGUAZAAgAHcAaQB0AGgAIAB0AGgAZQAgAGMAbwBuAHMAdQBtAHAAdABpAG8AbgAgAGEAbgBkACAAbABvAHMAcwBlAHMAIABvAGYAIABwAHUAcgBjAGgAYQBzAGUAZAAgAG8AcgAgAGEAYwBxAHUAaQByAGUAZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5ACAAcwBjAG8AcABlACAAMgAgAGEAbgBkACAAcwBjAG8AcABlACAAMwAgAGwAbwBjAGEAdABpAG8AbgAtAGIAYQBzAGUAZAAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAXAAiACkAKQA7AFwAbgBcAG4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEkAbgBkAGkAcgBlAGMAdAAgACgAcwBjAG8AcABlACAAMgAgAGEAbgBkACAAcwBjAG8AcABlACAAMwApACAAbABvAGMAYQB0AGkAbwBuAC0AYgBhAHMAZQBkACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGEAcwBzAG8AYwBpAGEAdABlAGQAIAB3AGkAdABoACAAdABoAGUAIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABhAG4AZAAgAGwAbwBzAHMAZQBzACAAbwBmACAAcAB1AHIAYwBoAGEAcwBlAGQAIABvAHIAIABhAGMAcQB1AGkAcgBlAGQAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAXAAiACkAKQA7AFwAbgBcAG4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABUAGEAYgBsAGUAIAAxAFwAIgApACkAOwBcAG4AXABuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMwAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALAAgAFQAZQByAHIAaQB0AG8AcgB5ACAAbwByACAAZwByAGkAZAAgAGQAZQBzAGMAcgBpAHAAdABpAG8AbgBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAyACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAcwAgACgAawBnACAAQwBPADIALQBlAC8AawBXAGgAKQBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAzACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAcwAgACgAawBnACAAQwBPADIALQBlAC8AawBXAGgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAGUAdwAgAFMAbwB1AHQAaAAgAFcAYQBsAGUAcwBcACIALAAgADAALgA2ADQALAAgADAALgAwADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAEMAVABcACIALAAgADAALgA2ADQALAAgADAALgAwADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIAAwAC4ANwA4ACwAIAAwAC4AMAA5ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgADAALgA2ADcALAAgADAALgAwADkAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AdQB0AGgAIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgADAALgAyADIALAAgADAALgAwADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAUwBvAHUAdABoACAAVwBlAHMAdAAgAEkAbgB0AGUAcgBjAG8AbgBuAGUAYwB0AGUAZAAgAFMAeQBzAHQAZQBtACAAKABTAFcASQBTACkAXAAiACwAIAAwAC4ANQAwACwAIAAwAC4AMAA2ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE4AbwByAHQAaAAgAFcAZQBzAHQAZQByAG4AIABJAG4AdABlAHIAYwBvAG4AbgBlAGMAdABlAGQAIABTAHkAcwB0AGUAbQAgACgATgBXAEkAUwApAFwAIgAsACAAMAAuADUANgAsACAAMAAuADAAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgADAALgAyADAALAAgADAALgAwADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AcgB0AGgAZQByAG4AIABUAGUAcgByAGkAdABvAHIAeQAgAC0AIABEAGEAcgB3AGkAbgAgAEsAYQB0AGgAZQByAGkAbgBlACAASQBuAHQAZQByAGMAbwBuAG4AZQBjAHQAZQBkACAAUwB5AHMAdABlAG0AIAAoAEQASwBJAFMAKQBcACIALAAgADAALgA1ADYALAAgADAALgAwADkAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAGEAdABpAG8AbgBhAGwAXAAiACwAIAAwAC4ANgAyACwAIAAwAC4AMAA3AFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAATgBTAFcAIABhAG4AZAAgAEEAQwBUACAAcwBwAGwAaQB0ACAAaQBuAHQAbwAgAHMAZQBwAGEAcgBhAHQAZQAgAHIAbwB3AHMALgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBSAGUAcwBpAGQAdQBhAGwAIABNAGkAeAAgAEYAYQBjAHQAbwByACAAZgBvAHIAIABtAGEAcgBrAGUAdAAtAGIAYQBzAGUAZAAgAGUAcQB1AGEAdABpAG8AbgBzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAIABzAGMAbwBwAGUAIAAyACAAYQBuAGQAIABzAGMAbwBwAGUAIAAzACAAbQBhAHIAawBlAHQALQBiAGEAcwBlAGQAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzAFwAIgApACkAOwBcAG4AXABuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAE0AYQByAGsAZQB0AEIAYQBzAGUAZABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFQAYQBiAGwAZQAgADIAYQAgAEkAbgBkAGkAcgBlAGMAdAAgACgAcwBjAG8AcABlACAAMgAgAGEAbgBkACAAcwBjAG8AcABlACAAMwApACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAcgBvAG0AIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABvAGYAIABwAHUAcgBjAGgAYQBzAGUAZAAgAG8AcgAgAGEAYwBxAHUAaQByAGUAZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQA6ACAAbQBhAHIAawBlAHQALQBiAGEAcwBlAGQAIABmAGEAYwB0AG8AcgBzACAAXAAiACkAKQA7AFwAbgBcAG4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATQBhAHIAawBlAHQAQgBhAHMAZQBkAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEEAYwBjAG8AdQBuAHQAcwAgAEYAYQBjAHQAbwByAHMAIAAyADAAMgA1ACAALQAgAFQAYQBiAGwAZQAgADIAYQBcACIAKQApADsAXABuAFwAbgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADUALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACwAIABUAGUAcgByAGkAdABvAHIAeQAgAG8AcgAgAGcAcgBpAGQAIABkAGUAcwBjAHIAaQBwAHQAaQBvAG4AXAAiACwAIABcACIAUwBjAG8AcABlACAAMgAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByAHMAIAAoAGsAZwAgAEMATwAyAC0AZQAvAGsAVwBoACkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMgAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByAHMAIAAoAGsAZwAgAEMATwAyAC0AZQAvAEcASgApAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADMAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgBzACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAGsAVwBoACkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMwAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByAHMAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATgBhAHQAaQBvAG4AYQBsAFwAIgAsACAAMAAuADgAMQAsACAAMgAyADYALAAgADAALgAxADAALAAgADIAOQBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATQBhAHIAawBlAHQAQgBhAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMQA0ADoAIABFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADEANAAuADEALgAxACAAUAB1AHIAYwBoAGEAcwBlAGQAIABFAGwAZQBjAHQAcgBpAGMAaQB0AHkAIAAoAEwAbwBjAGEAdABpAG8AbgAtAEIAYQBzAGUAZAApAFwAbgAxADQALgAxAC4AMgAgAFAAdQByAGMAaABhAHMAZQBkACAARQBsAGUAYwB0AHIAaQBjAGkAdAB5ACAAKABNAGEAcgBrAGUAdAAtAEIAYQBzAGUAZAApAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXABuAEwAbwBjAGEAdABpAG8AbgAtAGIAYQBzAGUAZAAgAFMAYwBvAHAAZQAgADIAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABwAHUAcgBjAGgAYQBzAGUAZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQBcAG4ARQBfADIAZQBsAGUAYwBcAG4AdAAgAEMATwAyAGUAXABuAEUAXwB7ADIALABlAGwAZQBjAH0APQBRAF8AewBlAGwAZQBjAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAMgAsAGUAbABlAGMAfQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4AUQBfAGUAbABlAGMAIAA9ACAAYQBtAG8AdQBuAHQAIABvAGYAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAIABwAHUAcgBjAGgAYQBzAGUAZAAgAGYAcgBvAG0AIAB0AGgAZQAgAGcAcgBpAGQAIAAoAGsAVwBoACkAXABuAEUARgBfADIAZQBsAGUAYwAgAD0AIABsAG8AYwBhAHQAaQBvAG4ALQBiAGEAcwBlAGQAIABTAGMAbwBwAGUAIAAyACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgACgAawBnACAAQwBPADIAZQAvAGsAVwBoACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUQBfAGUAbABlAGMALAAgAEUARgBfADIAZQBsAGUAYwAsAFwAbgAgACAAIAAgAFEAXwBlAGwAZQBjACAAKgAgAEUARgBfADIAZQBsAGUAYwAgACoAIAAxADAAIABeACAALQAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAbwBjAGEAdABpAG8AbgAtAGIAYQBzAGUAZAAgAFMAYwBvAHAAZQAgADIAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABwAHUAcgBjAGgAYQBzAGUAZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwAyAGUAbABlAGMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEANAAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsAMgAsAGUAbABlAGMAfQA9AFEAXwB7AGUAbABlAGMAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewAyACwAZQBsAGUAYwB9AFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMQBfAF8AMQBfAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AZQBsAGUAYwBcACIALAAgAFwAIgBhAG0AbwB1AG4AdAAgAG8AZgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQAgAHQAaABlACAAZwByAGkAZABcACIALAAgAFwAIgBrAFcAaABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfADIAZQBsAGUAYwBcACIALAAgAFwAIgBsAG8AYwBhAHQAaQBvAG4ALQBiAGEAcwBlAGQAIABTAGMAbwBwAGUAIAAyACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQBcACIALAAgAFwAIgBrAGcAIABDAE8AMgBlAC8AawBXAGgAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBnAFwAIgAsACAAXAAiAEcAcgBpAGQAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAIAB3AGEAcwAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMQBfAF8AMQBfAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAGQAZABlAGQAIABnACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYwBhAHAAdAB1AHIAZQAgAHcAaABpAGMAaAAgAGcAcgBpAGQAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAIAB3AGEAcwAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXABuAE0AYQByAGsAZQB0AC0AYgBhAHMAZQBkACAAUwBjAG8AcABlACAAMgAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHAAdQByAGMAaABhAHMAZQBkACAAZQBsAGUAYwB0AHIAaQBjAGkAdAB5AFwAbgBFAF8AMgBlAGwAZQBjAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBfAHsAMgAsAGUAbABlAGMAfQA9ACgAKABRAF8AewBlAGwAZQBjAH0AXABcAHQAaQBtAGUAcwAoADEALQAoAFIAUABQACsASgBSAFAAUAApACkAKQAtACgAKABSAEUAQwBfAHsAcwB1AHIAcgBlAG4AZABlAHIAZQBkAH0ALQBSAEUAQwBfAHsAbwBuAHMAaQB0AGUAfQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9ACkAKQBcAFwAdABpAG0AZQBzACAARQBGAF8AewBSAE0ARgAyACwAZQBsAGUAYwB9AFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBRAF8AZQBsAGUAYwAgAD0AIABhAG0AbwB1AG4AdAAgAG8AZgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQAgAHQAaABlACAAZwByAGkAZAAgACgAawBXAGgAKQBcAG4AUgBQAFAAIAA9ACAAUgBlAG4AZQB3AGEAYgBsAGUAIABQAG8AdwBlAHIAIABQAGUAcgBjAGUAbgB0AGEAZwBlACAAdQBuAGQAZQByACAAdABoAGUAIABMAGEAcgBnAGUALQBzAGMAYQBsAGUAIABSAGUAbgBlAHcAYQBiAGwAZQAgAEUAbgBlAHIAZwB5ACAAVABhAHIAZwBlAHQAIAAoAEwAUgBFAFQAKQAgAGYAbwByACAAdABoAGUAIABhAHAAcABsAGkAYwBhAGIAbABlACAAcABlAHIAaQBvAGQAIAAoAHAAZQByACAAYwBlAG4AdAApAFwAbgBKAFIAUABQACAAPQAgAGoAdQByAGkAcwBkAGkAYwB0AGkAbwBuAGEAbAAgAHIAZQBuAGUAdwBhAGIAbABlACAAcABvAHcAZQByACAAcABlAHIAYwBlAG4AdABhAGcAZQAgAGYAbwByACAAdABoAGUAIABhAHAAcABsAGkAYwBhAGIAbABlACAAcABlAHIAaQBvAGQAIAAoAG8AbgBsAHkAIABhAHAAcABsAGkAZQBzACAAdABvACAAdABoAGUAIABBAEMAVAApACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4AUgBFAEMAXwBzAHUAcgByAGUAbgBkAGUAcgBlAGQAIAA9ACAAbgB1AG0AYgBlAHIAIABvAGYAIABlAGwAaQBnAGkAYgBsAGUAIABSAGUAbgBlAHcAYQBiAGwAZQAgAEUAbgBlAHIAZwB5ACAAQwBlAHIAdABpAGYAaQBjAGEAdABlAHMAIAB2AG8AbAB1AG4AdABhAHIAaQBsAHkAIABzAHUAcgByAGUAbgBkAGUAcgBlAGQAIABpAG4AIAB0AGgAZQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAeQBlAGEAcgAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIAB0AG8AIABtAGUAZwBhAHcAYQB0AHQAIABoAG8AdQByAHMAIAAoAE0AVwBoACkAXABuAFIARQBDAF8AbwBuAHMAaQB0AGUAIAA9ACAAbgB1AG0AYgBlAHIAIABvAGYAIABlAGwAaQBnAGkAYgBsAGUAIABSAGUAbgBlAHcAYQBiAGwAZQAgAEUAbgBlAHIAZwB5ACAAQwBlAHIAdABpAGYAaQBjAGEAdABlAHMAIAB0AGgAYQB0ACAAaABhAHYAZQAgAGIAZQBlAG4AIABvAHIAIAB3AGkAbABsACAAYgBlACAAaQBzAHMAdQBlAGQAIABmAG8AcgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAcgBvAGQAdQBjAGUAZAAgAG8AbgAtAHMAaQB0AGUAIABkAHUAcgBpAG4AZwAgAHQAaABlACAAeQBlAGEAcgAgAGEAbgBkACAAYwBvAG4AcwB1AG0AZQBkACAAYgB5ACAAdABoAGUAIABlAG4AdABpAHQAeQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIAB0AG8AIABtAGUAZwBhAHcAYQB0AHQAIABoAG8AdQByAHMAIAAoAE0AVwBoACkAXABuAEUARgBfAFIATQBGADIAZQBsAGUAYwAgAD0AIABTAGMAbwBwAGUAIAAyACAAcgBlAHMAaQBkAHUAYQBsACAAbQBpAHgAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZQBsAGUAYwB0AHIAaQBjAGkAdAB5ACAAKABrAGcAIABDAE8AMgBlAC8AawBXAGgAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFEAXwBlAGwAZQBjACwAIABSAFAAUAAsACAASgBSAFAAUAAsACAAUgBFAEMAXwBzAHUAcgByAGUAbgBkAGUAcgBlAGQALAAgAFIARQBDAF8AbwBuAHMAaQB0AGUALAAgAEUARgBfAFIATQBGADIAZQBsAGUAYwAsAFwAbgAgACAAIAAgACgAKABRAF8AZQBsAGUAYwAgACoAIAAoADEAIAAtACAAKABSAFAAUAAgACsAIABKAFIAUABQACkAKQApACAALQAgACgAKABSAEUAQwBfAHMAdQByAHIAZQBuAGQAZQByAGUAZAAgAC0AIABSAEUAQwBfAG8AbgBzAGkAdABlACkAIAAqACAAMQAwACAAXgAgAC0AMwApACkAIAAqACAARQBGAF8AUgBNAEYAMgBlAGwAZQBjACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFEAXwBlAGwAZQBjACwAIABSAFAAUAAsACAASgBSAFAAUAAsACAAUgBFAEMAXwBzAHUAcgByAGUAbgBkAGUAcgBlAGQALAAgAFIARQBDAF8AbwBuAHMAaQB0AGUALAAgAEUARgBfAFIATQBGADIAZQBsAGUAYwAsAFwAbgAgACAAIAAgACgAKABRAF8AZQBsAGUAYwAgACoAIAAoADEAIAAtACAAKABSAFAAUAAgACsAIABKAFIAUABQACkAKQApACAALQAgACgAKABSAEUAQwBfAHMAdQByAHIAZQBuAGQAZQByAGUAZAAgAC0AIABSAEUAQwBfAG8AbgBzAGkAdABlACkAIAAqACAAMQAwACAAXgAgADMAKQApACAAKgAgAEUARgBfAFIATQBGADIAZQBsAGUAYwAgACoAIAAxADAAIABeACAALQAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAHIAawBlAHQALQBiAGEAcwBlAGQAIABTAGMAbwBwAGUAIAAyACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAcAB1AHIAYwBoAGEAcwBlAGQAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwAyAGUAbABlAGMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAxADQALgAxAC4AMgAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AewAyACwAZQBsAGUAYwB9AD0AKABRAF8AewBlAGwAZQBjAH0AIABcAFwAdABpAG0AZQBzACAAKAAxAC0AKABSAFAAUAArAEoAUgBQAFAAKQApACAALQAgACgAKABSAEUAQwBfAHsAcwB1AHIAcgBlAG4AZABlAHIAZQBkAH0ALQBSAEUAQwBfAHsAbwBuAHMAaQB0AGUAfQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9ACkAKQAgAFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AFIATQBGADIALABlAGwAZQBjAH0AIABcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBWAGEAcgBpAGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7ADIALABlAGwAZQBjAH0APQAoAFEAXwB7AGUAbABlAGMAfQAgAFwAXAB0AGkAbQBlAHMAIAAoADEALQAoAFIAUABQACsASgBSAFAAUAApACkAIAAtACAAKAAoAFIARQBDAF8AewBzAHUAcgByAGUAbgBkAGUAcgBlAGQAfQAtAFIARQBDAF8AewBvAG4AcwBpAHQAZQB9ACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsAMwB9ACkAKQAgAFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AFIATQBGADIALABlAGwAZQBjAH0AIABcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AZQBsAGUAYwBcACIALAAgAFwAIgBhAG0AbwB1AG4AdAAgAG8AZgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQAgAHQAaABlACAAZwByAGkAZABcACIALAAgAFwAIgBrAFcAaABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAUABQAFwAIgAsACAAXAAiAFIAZQBuAGUAdwBhAGIAbABlACAAUABvAHcAZQByACAAUABlAHIAYwBlAG4AdABhAGcAZQAgAHUAbgBkAGUAcgAgAHQAaABlACAATABhAHIAZwBlAC0AcwBjAGEAbABlACAAUgBlAG4AZQB3AGEAYgBsAGUAIABFAG4AZQByAGcAeQAgAFQAYQByAGcAZQB0ACAAKABMAFIARQBUACkAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgBSAFAAUABcACIALAAgAFwAIgBqAHUAcgBpAHMAZABpAGMAdABpAG8AbgBhAGwAIAByAGUAbgBlAHcAYQBiAGwAZQAgAHAAbwB3AGUAcgAgAHAAZQByAGMAZQBuAHQAYQBnAGUAIABmAG8AcgAgAHQAaABlACAAYQBwAHAAbABpAGMAYQBiAGwAZQAgAHAAZQByAGkAbwBkACAAKABBAEMAVAAgAG8AbgBsAHkAKQBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAEUAQwBfAHMAdQByAHIAZQBuAGQAZQByAGUAZABcACIALAAgAFwAIgBSAGUAbgBlAHcAYQBiAGwAZQAgAEUAbgBlAHIAZwB5ACAAQwBlAHIAdABpAGYAaQBjAGEAdABlAHMAIAB2AG8AbAB1AG4AdABhAHIAaQBsAHkAIABzAHUAcgByAGUAbgBkAGUAcgBlAGQAIABpAG4AIAB0AGgAZQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAeQBlAGEAcgBcACIALAAgAFwAIgBNAFcAaABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIARQBDAF8AbwBuAHMAaQB0AGUAXAAiACwAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABFAG4AZQByAGcAeQAgAEMAZQByAHQAaQBmAGkAYwBhAHQAZQBzACAAaQBzAHMAdQBlAGQAIABmAG8AcgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAcgBvAGQAdQBjAGUAZAAgAG8AbgAtAHMAaQB0AGUAIABkAHUAcgBpAG4AZwAgAHQAaABlACAAeQBlAGEAcgAgAGEAbgBkACAAYwBvAG4AcwB1AG0AZQBkACAAYgB5ACAAdABoAGUAIABlAG4AdABpAHQAeQBcACIALAAgAFwAIgBNAFcAaABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAFIATQBGADIAZQBsAGUAYwBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAyACAAcgBlAHMAaQBkAHUAYQBsACAAbQBpAHgAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZQBsAGUAYwB0AHIAaQBjAGkAdAB5AFwAIgAsACAAXAAiAGsAZwAgAEMATwAyAGUALwBrAFcAaABcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAIABcACIAcwB0AGEAdABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAASQBuACAAbwByAGQAZQByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAG0AZQBnAGEAdwBhAHQAdAAgAGgAbwB1AHIAcwAgAHQAbwAgAGsAaQBsAG8AdwBhAHQAdAAgAGgAbwB1AHIAcwAsACAAdABoAGUAIABSAEUAQwBfAHMAdQByAHIAZQBuAGQAZQByAGUAZAAgAGEAbgBkACAAUgBFAEMAXwBvAG4AcwBpAHQAZQAgAHYAYQByAGkAYQBiAGwAZQBzACAAYQByAGUAIABtAHUAbAB0AGkAcABsAGkAZQBkACAAYgB5ACAAMQAwAF4AMwAgAGkAbgBzAHQAZQBhAGQAIABvAGYAIAAxADAAXgAtADMALgBcACIAKQA7AFwAbgAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBUAGkAdABsAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBTAG8AdQByAGMAZQAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABfAEQAYQB0AGEAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATQBhAHIAawBlAHQAQgBhAHMAZQBkAF8AVABpAHQAbABlACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAE0AYQByAGsAZQB0AEIAYQBzAGUAZABfAFMAbwB1AHIAYwBlACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBEAGEAdABhACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMQBfAF8AMQBfAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMQBfAF8AMQBfAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFUAbgBpAHQAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAVgBhAHIAaQBhAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -14144,35 +14161,30 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACkAKgAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADIAKQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAEYARgBhAGwAcwBlACkAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwBlAGwAbAAsACAARABlAGwAaQBtAGkAdABlAHIALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEAXQAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgBdACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgBYAE0ATAAoAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAHQAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMAcwBcAHUAMAAwADMAZQBcACIAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFMAVQBCAFMAVABJAFQAVQBUAEUAKABDAGUAbABsACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADEALABcACIAXAAiACkALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABEAGUAbABpAG0AaQB0AGUAcgAsAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMAcwBcAHUAMAAwADMAZQBcACIAXABuACAAIAAgACAAIAAgACAAIAApACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAC8AdABcAHUAMAAwADMAZQBcACIALABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgAvAC8AcwBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAGEAdgBnAFQAZQBtAHAALABhAHYAZwBSAGEAaQBuACwAZgByAG8AcwB0AEQAYQB5AHMALABlAGwAZQB2ACwAbQBhAHAAXwBwAGUAdAAsAFwAbgAgACAAIAAgAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACwAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkALABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUABFAFQAQQByAHIAYQB5ACwAbQBhAHgAUABFAFQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AG0AYQBwAF8AcABlAHQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABQAEUAVABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AG0AYQBwAF8AcABlAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABBAEsARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgADEAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAE0AaQBuAEEAcgByAGEAeQAsACAATQBhAHgAQQByAHIAYQB5ACwAIABJAHQAZQBtAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AaQBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABJAHQAZQBtAEEAcgByAGEAeQAsACAAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAQwByAGkAdABlAHIAaQBhADEALAAgAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5ACwAIABRAHUAYQBuAHQAaQB0AHkALAAgAFsATQB1AGwAdABpAHAAbABpAGUAcgBdACwAIABbAEMAcgBpAHQAZQByAGkAYQAyAF0ALABbAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQBdACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgATQB1AGwAdABpAHAAbABpAGUAcgApACwAMQAsAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsAFwAbgAgACAAIAAgAHEAdQBhAG4AdABpAHQAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACoATQB1AGwAdABpAHAAbABpAGUAcgAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMQApACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADIALABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAcgBpAHQAZQByAGkAYQAyACkALAAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADIAKQApACwAXABuACAAIAAgACAAUwBVAE0AUABSAE8ARABVAEMAVAAoAGMAcgBpAHQAZQByAGkAYQAxACoAYwByAGkAdABlAHIAaQBhADIAKgBxAHUAYQBuAHQAaQB0AHkAKQBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjACAAUwApACwAXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAG4AZQB4AHQAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAUwApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBiACAAcwB0AGEAcgB0AHMAIABhAGYAdABlAHIAIABFACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUARQApACwAXABuACAAIAAgACAAIAAgACAAIABuACwATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAcgBzACwAUwBFAFEAVQBFAE4AQwBFACgAbgAsADEALABmAGkAcgBzAHQAWQBlAGEAcgAsADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMALABEAEEAVABFACgAeQByAHMALABtACwAZAApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzACwATQBBAFAAKABzAHQAYQByAHQAcwAsAFAAZQByAGkAbwBkAEUAbgBkACkALABcAG4AIAAgACAAIAAgACAAIAAgAHQAYQBnACwASQBGACgAcwB0AGEAcgB0AHMAPQBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXAAiACAAKABUAGgAaQBzACAAcgBlAHAAbwByAHQAaQBuAGcAIABjAHkAYwBsAGUAKQBcACIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzAFQAZQB4AHQALABUAEUAWABUACgAcwB0AGEAcgB0AHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzAFQAZQB4AHQALABUAEUAWABUACgAZQBuAGQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAXAAiACAAdABvACAAXAAiACAAXAB1ADAAMAAyADYAIABlAG4AZABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAHQAYQBnACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQBcAG4APQBMAEEATQBCAEQAQQAoAEYAdQBuAGMAdABpAG8AbgAsACAAVABFAFgAVABCAEUARgBPAFIARQAoAEYATwBSAE0AVQBMAEEAVABFAFgAVAAoAEYAdQBuAGMAdABpAG8AbgApACwAIABcACIAKABcACIAKQApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5ACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkALABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAA9AFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACAAPQAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5AD0AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkAPQBJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkAPQBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAFwAdQAwADAAMwBlADAALAAgADEALAAgADAAKQBcAG4AIAAgACAAIAApACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQAsACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAdQAwADAAMgA3AFwAIgAgAFwAdQAwADAAMgA2ACAAcwBoACAAXAB1ADAAMAAyADYAIABcACIAXAB1ADAAMAAyADcAIQBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsARABpAGYAZgBlAHIAZQBuAHQAUwBoAGUAZQB0AFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAxAF8AMgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADEALAAgADIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEMASABPAE8AUwBFAEMATwBMAFMAKABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALAAgADMALAAgADQAKQBcAG4AKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAATQBNAFMALAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFwAbgAgACAAIAAgACAAIAAgACAATQBFAEQASQBBAE4AKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ASQBuAGQAaQByAGUAYwB0ACAAKABzAGMAbwBwAGUAIAAyACAAYQBuAGQAIABzAGMAbwBwAGUAIAAzACkAIABsAG8AYwBhAHQAaQBvAG4ALQBiAGEAcwBlAGQAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAYQBzAHMAbwBjAGkAYQB0AGUAZAAgAHcAaQB0AGgAIAB0AGgAZQAgAGMAbwBuAHMAdQBtAHAAdABpAG8AbgAgAGEAbgBkACAAbABvAHMAcwBlAHMAIABvAGYAIABwAHUAcgBjAGgAYQBzAGUAZAAgAG8AcgAgAGEAYwBxAHUAaQByAGUAZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5ACAAcwBjAG8AcABlACAAMgAgAGEAbgBkACAAcwBjAG8AcABlACAAMwAgAGwAbwBjAGEAdABpAG8AbgAtAGIAYQBzAGUAZAAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAXAAiACkAKQA7AFwAbgBcAG4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEkAbgBkAGkAcgBlAGMAdAAgACgAcwBjAG8AcABlACAAMgAgAGEAbgBkACAAcwBjAG8AcABlACAAMwApACAAbABvAGMAYQB0AGkAbwBuAC0AYgBhAHMAZQBkACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGEAcwBzAG8AYwBpAGEAdABlAGQAIAB3AGkAdABoACAAdABoAGUAIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABhAG4AZAAgAGwAbwBzAHMAZQBzACAAbwBmACAAcAB1AHIAYwBoAGEAcwBlAGQAIABvAHIAIABhAGMAcQB1AGkAcgBlAGQAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAXAAiACkAKQA7AFwAbgBcAG4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABfAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABBAGMAYwBvAHUAbgB0AHMAIABGAGEAYwB0AG8AcgBzACAAMgAwADIANQAgAC0AIABUAGEAYgBsAGUAIAAxAFwAIgApACkAOwBcAG4AXABuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMwAsAFwAbgAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALAAgAFQAZQByAHIAaQB0AG8AcgB5ACAAbwByACAAZwByAGkAZAAgAGQAZQBzAGMAcgBpAHAAdABpAG8AbgBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAyACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAcwAgACgAawBnACAAQwBPADIALQBlAC8AawBXAGgAKQBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAzACAARQBtAGkAcwBzAGkAbwBuACAARgBhAGMAdABvAHIAcwAgACgAawBnACAAQwBPADIALQBlAC8AawBXAGgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAGUAdwAgAFMAbwB1AHQAaAAgAFcAYQBsAGUAcwBcACIALAAgADAALgA2ADQALAAgADAALgAwADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAEMAVABcACIALAAgADAALgA2ADQALAAgADAALgAwADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIAAwAC4ANwA4ACwAIAAwAC4AMAA5ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgADAALgA2ADcALAAgADAALgAwADkAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AdQB0AGgAIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgADAALgAyADIALAAgADAALgAwADQAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAUwBvAHUAdABoACAAVwBlAHMAdAAgAEkAbgB0AGUAcgBjAG8AbgBuAGUAYwB0AGUAZAAgAFMAeQBzAHQAZQBtACAAKABTAFcASQBTACkAXAAiACwAIAAwAC4ANQAwACwAIAAwAC4AMAA2ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE4AbwByAHQAaAAgAFcAZQBzAHQAZQByAG4AIABJAG4AdABlAHIAYwBvAG4AbgBlAGMAdABlAGQAIABTAHkAcwB0AGUAbQAgACgATgBXAEkAUwApAFwAIgAsACAAMAAuADUANgAsACAAMAAuADAAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgADAALgAyADAALAAgADAALgAwADMAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AcgB0AGgAZQByAG4AIABUAGUAcgByAGkAdABvAHIAeQAgAC0AIABEAGEAcgB3AGkAbgAgAEsAYQB0AGgAZQByAGkAbgBlACAASQBuAHQAZQByAGMAbwBuAG4AZQBjAHQAZQBkACAAUwB5AHMAdABlAG0AIAAoAEQASwBJAFMAKQBcACIALAAgADAALgA1ADYALAAgADAALgAwADkAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBOAGEAdABpAG8AbgBhAGwAXAAiACwAIAAwAC4ANgAyACwAIAAwAC4AMAA3AFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAATgBTAFcAIABhAG4AZAAgAEEAQwBUACAAcwBwAGwAaQB0ACAAaQBuAHQAbwAgAHMAZQBwAGEAcgBhAHQAZQAgAHIAbwB3AHMALgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBSAGUAcwBpAGQAdQBhAGwAIABNAGkAeAAgAEYAYQBjAHQAbwByACAAZgBvAHIAIABtAGEAcgBrAGUAdAAtAGIAYQBzAGUAZAAgAGUAcQB1AGEAdABpAG8AbgBzAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBUAGkAdABsAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAIABzAGMAbwBwAGUAIAAyACAAYQBuAGQAIABzAGMAbwBwAGUAIAAzACAAbQBhAHIAawBlAHQALQBiAGEAcwBlAGQAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzAFwAIgApACkAOwBcAG4AXABuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAE0AYQByAGsAZQB0AEIAYQBzAGUAZABfAEQAZQBzAGMAcgBpAHAAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFQAYQBiAGwAZQAgADIAYQAgAEkAbgBkAGkAcgBlAGMAdAAgACgAcwBjAG8AcABlACAAMgAgAGEAbgBkACAAcwBjAG8AcABlACAAMwApACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAcgBvAG0AIABjAG8AbgBzAHUAbQBwAHQAaQBvAG4AIABvAGYAIABwAHUAcgBjAGgAYQBzAGUAZAAgAG8AcgAgAGEAYwBxAHUAaQByAGUAZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQA6ACAAbQBhAHIAawBlAHQALQBiAGEAcwBlAGQAIABmAGEAYwB0AG8AcgBzACAAXAAiACkAKQA7AFwAbgBcAG4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATQBhAHIAawBlAHQAQgBhAHMAZQBkAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEEAYwBjAG8AdQBuAHQAcwAgAEYAYQBjAHQAbwByAHMAIAAyADAAMgA1ACAALQAgAFQAYQBiAGwAZQAgADIAYQBcACIAKQApADsAXABuAFwAbgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBEAGEAdABhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADUALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACwAIABUAGUAcgByAGkAdABvAHIAeQAgAG8AcgAgAGcAcgBpAGQAIABkAGUAcwBjAHIAaQBwAHQAaQBvAG4AXAAiACwAIABcACIAUwBjAG8AcABlACAAMgAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByAHMAIAAoAGsAZwAgAEMATwAyAC0AZQAvAGsAVwBoACkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMgAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByAHMAIAAoAGsAZwAgAEMATwAyAC0AZQAvAEcASgApAFwAIgAsACAAXAAiAFMAYwBvAHAAZQAgADMAIABFAG0AaQBzAHMAaQBvAG4AIABGAGEAYwB0AG8AcgBzACAAKABrAGcAIABDAE8AMgAgAC0AIABlACAALwAgAGsAVwBoACkAXAAiACwAIABcACIAUwBjAG8AcABlACAAMwAgAEUAbQBpAHMAcwBpAG8AbgAgAEYAYQBjAHQAbwByAHMAIAAoAGsAZwAgAEMATwAyACAALQAgAGUAIAAvACAARwBKACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATgBhAHQAaQBvAG4AYQBsAFwAIgAsACAAMAAuADgAMQAsACAAMgAyADYALAAgADAALgAxADAALAAgADIAOQBcAG4AIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgApACkAKQA7AFwAbgBcAG4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATQBhAHIAawBlAHQAQgBhAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMQA0ADoAIABFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADEANAAuADEALgAxACAAUAB1AHIAYwBoAGEAcwBlAGQAIABFAGwAZQBjAHQAcgBpAGMAaQB0AHkAIAAoAEwAbwBjAGEAdABpAG8AbgAtAEIAYQBzAGUAZAApAFwAbgAxADQALgAxAC4AMgAgAFAAdQByAGMAaABhAHMAZQBkACAARQBsAGUAYwB0AHIAaQBjAGkAdAB5ACAAKABNAGEAcgBrAGUAdAAtAEIAYQBzAGUAZAApAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXABuAEwAbwBjAGEAdABpAG8AbgAtAGIAYQBzAGUAZAAgAFMAYwBvAHAAZQAgADIAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABwAHUAcgBjAGgAYQBzAGUAZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQBcAG4ARQBfADIAZQBsAGUAYwBcAG4AdAAgAEMATwAyAGUAXABuAEUAXwB7ADIALABlAGwAZQBjAH0APQBRAF8AewBlAGwAZQBjAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAMgAsAGUAbABlAGMAfQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4AUQBfAGUAbABlAGMAIAA9ACAAYQBtAG8AdQBuAHQAIABvAGYAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAIABwAHUAcgBjAGgAYQBzAGUAZAAgAGYAcgBvAG0AIAB0AGgAZQAgAGcAcgBpAGQAIAAoAGsAVwBoACkAXABuAEUARgBfADIAZQBsAGUAYwAgAD0AIABsAG8AYwBhAHQAaQBvAG4ALQBiAGEAcwBlAGQAIABTAGMAbwBwAGUAIAAyACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgACgAawBnACAAQwBPADIAZQAvAGsAVwBoACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUQBfAGUAbABlAGMALAAgAEUARgBfADIAZQBsAGUAYwAsAFwAbgAgACAAIAAgAFEAXwBlAGwAZQBjACAAKgAgAEUARgBfADIAZQBsAGUAYwAgACoAIAAxADAAIABeACAALQAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAbwBjAGEAdABpAG8AbgAtAGIAYQBzAGUAZAAgAFMAYwBvAHAAZQAgADIAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABwAHUAcgBjAGgAYQBzAGUAZAAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwAyAGUAbABlAGMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEANAAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsAMgAsAGUAbABlAGMAfQA9AFEAXwB7AGUAbABlAGMAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewAyACwAZQBsAGUAYwB9AFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMQBfAF8AMQBfAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AZQBsAGUAYwBcACIALAAgAFwAIgBhAG0AbwB1AG4AdAAgAG8AZgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQAgAHQAaABlACAAZwByAGkAZABcACIALAAgAFwAIgBrAFcAaABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfADIAZQBsAGUAYwBcACIALAAgAFwAIgBsAG8AYwBhAHQAaQBvAG4ALQBiAGEAcwBlAGQAIABTAGMAbwBwAGUAIAAyACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQBcACIALAAgAFwAIgBrAGcAIABDAE8AMgBlAC8AawBXAGgAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBnAFwAIgAsACAAXAAiAEcAcgBpAGQAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAIAB3AGEAcwAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMQBfAF8AMQBfAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAGQAZABlAGQAIABnACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYwBhAHAAdAB1AHIAZQAgAHcAaABpAGMAaAAgAGcAcgBpAGQAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAIAB3AGEAcwAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQBcACIAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXABuAE0AYQByAGsAZQB0AC0AYgBhAHMAZQBkACAAUwBjAG8AcABlACAAMgAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHAAdQByAGMAaABhAHMAZQBkACAAZQBsAGUAYwB0AHIAaQBjAGkAdAB5AFwAbgBFAF8AMgBlAGwAZQBjAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBfAHsAMgAsAGUAbABlAGMAfQA9ACgAKABRAF8AewBlAGwAZQBjAH0AXABcAHQAaQBtAGUAcwAoADEALQAoAFIAUABQACsASgBSAFAAUAApACkAKQAtACgAKABSAEUAQwBfAHsAcwB1AHIAcgBlAG4AZABlAHIAZQBkAH0ALQBSAEUAQwBfAHsAbwBuAHMAaQB0AGUAfQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9ACkAKQBcAFwAdABpAG0AZQBzACAARQBGAF8AewBSAE0ARgAyACwAZQBsAGUAYwB9AFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBRAF8AZQBsAGUAYwAgAD0AIABhAG0AbwB1AG4AdAAgAG8AZgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQAgAHQAaABlACAAZwByAGkAZAAgACgAawBXAGgAKQBcAG4AUgBQAFAAIAA9ACAAUgBlAG4AZQB3AGEAYgBsAGUAIABQAG8AdwBlAHIAIABQAGUAcgBjAGUAbgB0AGEAZwBlACAAdQBuAGQAZQByACAAdABoAGUAIABMAGEAcgBnAGUALQBzAGMAYQBsAGUAIABSAGUAbgBlAHcAYQBiAGwAZQAgAEUAbgBlAHIAZwB5ACAAVABhAHIAZwBlAHQAIAAoAEwAUgBFAFQAKQAgAGYAbwByACAAdABoAGUAIABhAHAAcABsAGkAYwBhAGIAbABlACAAcABlAHIAaQBvAGQAIAAoAHAAZQByACAAYwBlAG4AdAApAFwAbgBKAFIAUABQACAAPQAgAGoAdQByAGkAcwBkAGkAYwB0AGkAbwBuAGEAbAAgAHIAZQBuAGUAdwBhAGIAbABlACAAcABvAHcAZQByACAAcABlAHIAYwBlAG4AdABhAGcAZQAgAGYAbwByACAAdABoAGUAIABhAHAAcABsAGkAYwBhAGIAbABlACAAcABlAHIAaQBvAGQAIAAoAG8AbgBsAHkAIABhAHAAcABsAGkAZQBzACAAdABvACAAdABoAGUAIABBAEMAVAApACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4AUgBFAEMAXwBzAHUAcgByAGUAbgBkAGUAcgBlAGQAIAA9ACAAbgB1AG0AYgBlAHIAIABvAGYAIABlAGwAaQBnAGkAYgBsAGUAIABSAGUAbgBlAHcAYQBiAGwAZQAgAEUAbgBlAHIAZwB5ACAAQwBlAHIAdABpAGYAaQBjAGEAdABlAHMAIAB2AG8AbAB1AG4AdABhAHIAaQBsAHkAIABzAHUAcgByAGUAbgBkAGUAcgBlAGQAIABpAG4AIAB0AGgAZQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAeQBlAGEAcgAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIAB0AG8AIABtAGUAZwBhAHcAYQB0AHQAIABoAG8AdQByAHMAIAAoAE0AVwBoACkAXABuAFIARQBDAF8AbwBuAHMAaQB0AGUAIAA9ACAAbgB1AG0AYgBlAHIAIABvAGYAIABlAGwAaQBnAGkAYgBsAGUAIABSAGUAbgBlAHcAYQBiAGwAZQAgAEUAbgBlAHIAZwB5ACAAQwBlAHIAdABpAGYAaQBjAGEAdABlAHMAIAB0AGgAYQB0ACAAaABhAHYAZQAgAGIAZQBlAG4AIABvAHIAIAB3AGkAbABsACAAYgBlACAAaQBzAHMAdQBlAGQAIABmAG8AcgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAcgBvAGQAdQBjAGUAZAAgAG8AbgAtAHMAaQB0AGUAIABkAHUAcgBpAG4AZwAgAHQAaABlACAAeQBlAGEAcgAgAGEAbgBkACAAYwBvAG4AcwB1AG0AZQBkACAAYgB5ACAAdABoAGUAIABlAG4AdABpAHQAeQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIAB0AG8AIABtAGUAZwBhAHcAYQB0AHQAIABoAG8AdQByAHMAIAAoAE0AVwBoACkAXABuAEUARgBfAFIATQBGADIAZQBsAGUAYwAgAD0AIABTAGMAbwBwAGUAIAAyACAAcgBlAHMAaQBkAHUAYQBsACAAbQBpAHgAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZQBsAGUAYwB0AHIAaQBjAGkAdAB5ACAAKABrAGcAIABDAE8AMgBlAC8AawBXAGgAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFEAXwBlAGwAZQBjACwAIABSAFAAUAAsACAASgBSAFAAUAAsACAAUgBFAEMAXwBzAHUAcgByAGUAbgBkAGUAcgBlAGQALAAgAFIARQBDAF8AbwBuAHMAaQB0AGUALAAgAEUARgBfAFIATQBGADIAZQBsAGUAYwAsAFwAbgAgACAAIAAgACgAKABRAF8AZQBsAGUAYwAgACoAIAAoADEAIAAtACAAKABSAFAAUAAgACsAIABKAFIAUABQACkAKQApACAALQAgACgAKABSAEUAQwBfAHMAdQByAHIAZQBuAGQAZQByAGUAZAAgAC0AIABSAEUAQwBfAG8AbgBzAGkAdABlACkAIAAqACAAMQAwACAAXgAgAC0AMwApACkAIAAqACAARQBGAF8AUgBNAEYAMgBlAGwAZQBjACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFEAXwBlAGwAZQBjACwAIABSAFAAUAAsACAASgBSAFAAUAAsACAAUgBFAEMAXwBzAHUAcgByAGUAbgBkAGUAcgBlAGQALAAgAFIARQBDAF8AbwBuAHMAaQB0AGUALAAgAEUARgBfAFIATQBGADIAZQBsAGUAYwAsAFwAbgAgACAAIAAgACgAKABRAF8AZQBsAGUAYwAgACoAIAAoADEAIAAtACAAKABSAFAAUAAgACsAIABKAFIAUABQACkAKQApACAALQAgACgAKABSAEUAQwBfAHMAdQByAHIAZQBuAGQAZQByAGUAZAAgAC0AIABSAEUAQwBfAG8AbgBzAGkAdABlACkAIAAqACAAMQAwACAAXgAgADMAKQApACAAKgAgAEUARgBfAFIATQBGADIAZQBsAGUAYwAgACoAIAAxADAAIABeACAALQAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAHIAawBlAHQALQBiAGEAcwBlAGQAIABTAGMAbwBwAGUAIAAyACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAcAB1AHIAYwBoAGEAcwBlAGQAIABlAGwAZQBjAHQAcgBpAGMAaQB0AHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwAyAGUAbABlAGMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAxADQALgAxAC4AMgAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AewAyACwAZQBsAGUAYwB9AD0AKABRAF8AewBlAGwAZQBjAH0AIABcAFwAdABpAG0AZQBzACAAKAAxAC0AKABSAFAAUAArAEoAUgBQAFAAKQApACAALQAgACgAKABSAEUAQwBfAHsAcwB1AHIAcgBlAG4AZABlAHIAZQBkAH0ALQBSAEUAQwBfAHsAbwBuAHMAaQB0AGUAfQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9ACkAKQAgAFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AFIATQBGADIALABlAGwAZQBjAH0AIABcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBWAGEAcgBpAGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7ADIALABlAGwAZQBjAH0APQAoAFEAXwB7AGUAbABlAGMAfQAgAFwAXAB0AGkAbQBlAHMAIAAoADEALQAoAFIAUABQACsASgBSAFAAUAApACkAIAAtACAAKAAoAFIARQBDAF8AewBzAHUAcgByAGUAbgBkAGUAcgBlAGQAfQAtAFIARQBDAF8AewBvAG4AcwBpAHQAZQB9ACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsAMwB9ACkAKQAgAFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AFIATQBGADIALABlAGwAZQBjAH0AIABcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAF8AZQBsAGUAYwBcACIALAAgAFwAIgBhAG0AbwB1AG4AdAAgAG8AZgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAdQByAGMAaABhAHMAZQBkACAAZgByAG8AbQAgAHQAaABlACAAZwByAGkAZABcACIALAAgAFwAIgBrAFcAaABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAUABQAFwAIgAsACAAXAAiAFIAZQBuAGUAdwBhAGIAbABlACAAUABvAHcAZQByACAAUABlAHIAYwBlAG4AdABhAGcAZQAgAHUAbgBkAGUAcgAgAHQAaABlACAATABhAHIAZwBlAC0AcwBjAGEAbABlACAAUgBlAG4AZQB3AGEAYgBsAGUAIABFAG4AZQByAGcAeQAgAFQAYQByAGcAZQB0ACAAKABMAFIARQBUACkAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgBSAFAAUABcACIALAAgAFwAIgBqAHUAcgBpAHMAZABpAGMAdABpAG8AbgBhAGwAIAByAGUAbgBlAHcAYQBiAGwAZQAgAHAAbwB3AGUAcgAgAHAAZQByAGMAZQBuAHQAYQBnAGUAIABmAG8AcgAgAHQAaABlACAAYQBwAHAAbABpAGMAYQBiAGwAZQAgAHAAZQByAGkAbwBkACAAKABBAEMAVAAgAG8AbgBsAHkAKQBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAEUAQwBfAHMAdQByAHIAZQBuAGQAZQByAGUAZABcACIALAAgAFwAIgBSAGUAbgBlAHcAYQBiAGwAZQAgAEUAbgBlAHIAZwB5ACAAQwBlAHIAdABpAGYAaQBjAGEAdABlAHMAIAB2AG8AbAB1AG4AdABhAHIAaQBsAHkAIABzAHUAcgByAGUAbgBkAGUAcgBlAGQAIABpAG4AIAB0AGgAZQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAeQBlAGEAcgBcACIALAAgAFwAIgBNAFcAaABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIARQBDAF8AbwBuAHMAaQB0AGUAXAAiACwAIABcACIAUgBlAG4AZQB3AGEAYgBsAGUAIABFAG4AZQByAGcAeQAgAEMAZQByAHQAaQBmAGkAYwBhAHQAZQBzACAAaQBzAHMAdQBlAGQAIABmAG8AcgAgAGUAbABlAGMAdAByAGkAYwBpAHQAeQAgAHAAcgBvAGQAdQBjAGUAZAAgAG8AbgAtAHMAaQB0AGUAIABkAHUAcgBpAG4AZwAgAHQAaABlACAAeQBlAGEAcgAgAGEAbgBkACAAYwBvAG4AcwB1AG0AZQBkACAAYgB5ACAAdABoAGUAIABlAG4AdABpAHQAeQBcACIALAAgAFwAIgBNAFcAaABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAFIATQBGADIAZQBsAGUAYwBcACIALAAgAFwAIgBTAGMAbwBwAGUAIAAyACAAcgBlAHMAaQBkAHUAYQBsACAAbQBpAHgAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZQBsAGUAYwB0AHIAaQBjAGkAdAB5AFwAIgAsACAAXAAiAGsAZwAgAEMATwAyAGUALwBrAFcAaABcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAIABcACIAcwB0AGEAdABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAASQBuACAAbwByAGQAZQByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAG0AZQBnAGEAdwBhAHQAdAAgAGgAbwB1AHIAcwAgAHQAbwAgAGsAaQBsAG8AdwBhAHQAdAAgAGgAbwB1AHIAcwAsACAAdABoAGUAIABSAEUAQwBfAHMAdQByAHIAZQBuAGQAZQByAGUAZAAgAGEAbgBkACAAUgBFAEMAXwBvAG4AcwBpAHQAZQAgAHYAYQByAGkAYQBiAGwAZQBzACAAYQByAGUAIABtAHUAbAB0AGkAcABsAGkAZQBkACAAYgB5ACAAMQAwAF4AMwAgAGkAbgBzAHQAZQBhAGQAIABvAGYAIAAxADAAXgAtADMALgBcACIAKQA7AFwAbgAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBUAGkAdABsAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBTAG8AdQByAGMAZQAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABfAEQAYQB0AGEAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4ARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBjAG8AcABlADIAUwBjAG8AcABlADMATQBhAHIAawBlAHQAQgBhAHMAZQBkAF8AVABpAHQAbABlACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBEAGUAcwBjAHIAaQBwAHQAaQBvAG4AIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAYwBvAHAAZQAyAFMAYwBvAHAAZQAzAE0AYQByAGsAZQB0AEIAYQBzAGUAZABfAFMAbwB1AHIAYwBlACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBEAGEAdABhACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBTAGMAbwBwAGUAMgBTAGMAbwBwAGUAMwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMQBfAF8AMQBfAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMQBfAF8AMQBfAEwAbwBjAGEAdABpAG8AbgBCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADEAXwBfADEAXwBMAG8AYwBhAHQAaQBvAG4AQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAxAF8AXwAxAF8ATABvAGMAYQB0AGkAbwBuAEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFUAbgBpAHQAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBsAGUAYwB0AHIAaQBjAGkAdAB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADQAXwAxAF8AMgBfAF8AMQBfAE0AYQByAGsAZQB0AEIAYQBzAGUAZABTAGMAbwBwAGUARQBsAGUAYwB0AHIAaQBjAGkAdAB5AEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAGwAZQBjAHQAcgBpAGMAaQB0AHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEANABfADEAXwAyAF8AXwAxAF8ATQBhAHIAawBlAHQAQgBhAHMAZQBkAFMAYwBvAHAAZQBFAGwAZQBjAHQAcgBpAGMAaQB0AHkARQBtAGkAcwBzAGkAbwBuAHMAVgBhAHIAaQBhAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbABlAGMAdAByAGkAYwBpAHQAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQA0AF8AMQBfADIAXwBfADEAXwBNAGEAcgBrAGUAdABCAGEAcwBlAGQAUwBjAG8AcABlAEUAbABlAGMAdAByAGkAYwBpAHQAeQBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14191,21 +14203,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>